<commit_message>
task130 hardening loop 1: move-on lists on Part 3 need on each round day from the household members (the case record lags children reaching 10 and 16), rounds on the third Monday, exact-size lists, units sized on the 1 April need; answer 52 units (0/10/18/24)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task130/golden/tenter_house_replacement_units.xlsx
+++ b/task130/golden/tenter_house_replacement_units.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>374.93</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>2624.51</v>
+        <v>3749.3</v>
       </c>
     </row>
     <row r="7">
@@ -569,19 +569,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>444.06</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>8881.200000000001</v>
+        <v>7993.08</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C8" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>532.08</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>10109.52</v>
+        <v>12769.92</v>
       </c>
     </row>
     <row r="9">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>21615.23</v>
+        <v>24512.3</v>
       </c>
     </row>
     <row r="10"/>
@@ -633,28 +633,28 @@
         </is>
       </c>
       <c r="F11" s="8" t="n">
-        <v>21615</v>
+        <v>24512</v>
       </c>
     </row>
     <row r="12"/>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Households and units are whole numbers. Bedrooms are the need as assessed at 18 September 2026 (closure procedure, point 5); 4+ means four or more.</t>
+          <t>Households and units are whole numbers. Each household is counted under the unit it will need on 1 April 2027 under Part 3 of the allocations scheme, from the people on its application on 30 September 2026 (closure procedure, point 5); 4+ means four or more.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Expected households: those the move-on plan's lets (revised 14 September 2026) do not reach by 31 March. Move-on lets go to every household owed the main duty, in or out of TA, by duty date within the bedroom need, case reference breaking ties; the lets log since April 2018 follows that order without exception.</t>
+          <t>Expected households: those the move-on plan's lets (revised 14 September 2026) do not reach by 31 March. Each month's homes go in the round held on the third Monday of the month before, to every household owed the main duty, in or out of TA, by duty date within the bedrooms it needs on the round day (scheme 3.4 and 6.4). Needs are worked out from the household members for each round; the bedroom need on the case record is only reassessed at a decision, a reported birth, a move or an offer.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>October lets already accepted are inside the plan's October figures and are not counted again.</t>
+          <t>October's lets were all offered in the round of 21 September and are counted once. No homes with five or more bedrooms are planned, so households needing five or more stay on that list.</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>By bedroom need. 30 September 2026 is the extract position; the months follow the revised move-on plan.</t>
+          <t>By the size of unit each household will need on 1 April 2027. 30 September 2026 is the extract position; the months follow the revised move-on plan.</t>
         </is>
       </c>
     </row>
@@ -759,16 +759,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
         <v>20</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -787,25 +787,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D6" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E6" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F6" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G6" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -815,25 +815,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E7" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F7" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G7" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H7" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -843,25 +843,25 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>31</v>
+      </c>
+      <c r="C8" t="n">
+        <v>31</v>
+      </c>
+      <c r="D8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" t="n">
+        <v>29</v>
+      </c>
+      <c r="G8" t="n">
         <v>26</v>
       </c>
-      <c r="C8" t="n">
-        <v>26</v>
-      </c>
-      <c r="D8" t="n">
-        <v>25</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="H8" t="n">
         <v>24</v>
-      </c>
-      <c r="F8" t="n">
-        <v>23</v>
-      </c>
-      <c r="G8" t="n">
-        <v>21</v>
-      </c>
-      <c r="H8" t="n">
-        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -871,25 +871,25 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>